<commit_message>
Fix classification bug: merge D03 into D53 (same problem type)
D03 (1 question, p006_q14) and D53 (3 questions) were both
log_a(linear)>k basic logarithmic inequalities, tách nhầm thành 2 mã dạng
khác nhau. Merged p006_q14 into D53 and added it to the pilot generator,
dropping the total unique problem-type count from 94 to 93.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions/mu_logarit_extraction/Mu_Logarit_112_cau_phan_dang.xlsx
+++ b/data/questions/mu_logarit_extraction/Mu_Logarit_112_cau_phan_dang.xlsx
@@ -567,12 +567,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D53</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Giải bất phương trình lôgarit cơ bản dạng log_a(f(x))&gt;k, f(x) bậc nhất</t>
+          <t>Giải bất phương trình lôgarit cơ bản dạng log_a(f(x))&gt;k</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">

</xml_diff>